<commit_message>
site build 2026-10-08 21:29
</commit_message>
<xml_diff>
--- a/models/sovereigns/Cote_d_Ivoire_Sovereign_Model.xlsx
+++ b/models/sovereigns/Cote_d_Ivoire_Sovereign_Model.xlsx
@@ -700,7 +700,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Institut National de la Statistique (IHPC)</t>
+          <t>INS Cote d'Ivoire, IHPC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>01-Jun-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -784,12 +784,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>01-Jun-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Central government debt</t>
+          <t>Government debt, projection; WAEMU ceiling 70%</t>
         </is>
       </c>
     </row>
@@ -826,17 +826,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>2026 budget</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IMF / Ministry of Finance (budgeted deficit)</t>
+          <t>IMF / Ministry of Finance</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>30-Jun-26</t>
+          <t>01-Jun-26</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -921,11 +921,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -956,11 +952,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1071,7 +1063,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>112.115</v>
+        <v>112.1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1093,11 +1085,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1263,11 +1251,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EFF/ECF (40-month, US$3.5B) and RSF (US$1.3B); final reviews completed Jun-26</t>
+          <t>EFF/ECF (US$3.5B) and RSF (US$1.3B), final reviews completed Jun-26</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4.8</v>
+        <v>3.5</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1326,9 +1314,15 @@
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="n">
+        <v>112.1</v>
+      </c>
       <c r="D2" s="2" t="n"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1345,7 +1339,7 @@
       <c r="D3" s="2" t="n"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>IMF, 30-Jun-26</t>
+          <t>IMF, Jun-26</t>
         </is>
       </c>
     </row>
@@ -1367,9 +1361,15 @@
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="n">
+        <v>-1.1</v>
+      </c>
       <c r="D5" s="2" t="n"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IMF / Ministry of Finance, 30-Jun-26 (2025 outturn at WAEMU 3.0% ceiling; 2028F is the commitment to return to the ceiling)</t>
+          <t>IMF / Ministry of Finance, Jun-26</t>
         </is>
       </c>
     </row>
@@ -1418,7 +1418,7 @@
       <c r="D8" s="2" t="n"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF / Ministry of Finance, 30-Jun-26</t>
+          <t>IMF / Ministry of Finance, Jun-26</t>
         </is>
       </c>
     </row>

</xml_diff>